<commit_message>
moved default open sheet to samples
</commit_message>
<xml_diff>
--- a/src/ESM.xlsx
+++ b/src/ESM.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58B0938-62BA-6941-B525-5FB3A33BADC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="23040" windowHeight="13560" activeTab="3" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="23040" windowHeight="13560" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
   <sheets>
     <sheet name="Samples" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
update template: remove name, added validations
</commit_message>
<xml_diff>
--- a/src/ESM.xlsx
+++ b/src/ESM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58B0938-62BA-6941-B525-5FB3A33BADC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C73AF8C-C2F1-E44B-81B1-8BEB85550543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="23040" windowHeight="13560" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
   <sheets>
     <sheet name="Samples" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>Plate</t>
   </si>
@@ -454,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2569E313-B3CC-438F-A253-EA0F3E8D819B}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" style="1" bestFit="1" customWidth="1"/>
@@ -463,7 +463,7 @@
     <col min="4" max="4" width="14.5" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -481,13 +481,22 @@
       </c>
       <c r="F1" t="s">
         <v>2</v>
-      </c>
-      <c r="G1" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Plate brand" prompt="The brand of plate reader used for the data. If Samples::Type is not plate reader, this can be left blank." sqref="D2:D1048576" xr:uid="{F795587E-0606-8D47-AA35-A77937E6BFD0}">
+      <formula1>"BioTek, Tecan, BMG, SpectraMax, Generic"</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Type" prompt="The type of experimental data. Either &quot;plate reader&quot; for any plate reader file, or &quot;flow&quot; for flow cytometry fcs files." sqref="A2:A1048576" xr:uid="{CF35B5DA-5768-0E4F-878A-C64AE48DF9B0}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Data Location" prompt="The file location of the experimental data. It should either be an absolute file path, or relative to the directory from which esm translate is called. If Samples::Type=&quot;flow&quot;, this can be a directory of fcs files." sqref="B2:B1048576" xr:uid="{C349ED61-BB07-3C40-8A36-DD5340FD2263}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Channels" prompt="The channels to translate into the esm file. Any channels not specified will not be included. If blank, all channels will be included. Available channels can be found with esm summarise. Multiple channels can be provided as a comma-separated list." sqref="C2:C1048576" xr:uid="{551D77D5-3392-5345-AFA9-BEC77E06FD7B}"/>
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Plate" prompt="The plate number used in ESM to refer to this data. Must be a positive whole number. For example, if Samples::Plate=5, this data can be referred to as the wells of plate_05 in ESM." sqref="E2:E1048576" xr:uid="{107CB822-50EF-4C42-B564-6339739ADB7F}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Well" prompt="The well used to access the data. If the data defines multiple wells (e.g. Samples::Type=&quot;plate reader&quot; or Samples::Data Location refers to a directory of fcs files), this should be left blank. Otherwise, it should describe the well name, A1, B6, etc." sqref="F2:F1048576" xr:uid="{6B1A893B-FCED-AC4A-9788-458982851B69}"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -510,6 +519,10 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Channel Map::Channel" prompt="The original channel name as given in Samples::Channels and by esm summarise." sqref="A2:A1048576" xr:uid="{03B4CC33-3D41-214B-B1F0-944AC5F72A89}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Channel Map::New name" prompt="The new name for the channel. ESM will override all instances of the Channel Map::Channel name with this name." sqref="B2:B1048576" xr:uid="{1C30423D-F4B1-B243-89E0-84AB035D067E}"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -532,6 +545,10 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Groups::Name" prompt="The name of the group. This is the name that will be used to refer to the group in ESM. It should only contain alphanumeric characters and underscores, starting with a letter." sqref="A2:A1048576" xr:uid="{4FADBE0B-141D-5748-9249-7B04C7BBB1DF}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Groups::Samples" prompt="The wells that are contained within the group as a comma separated list. A short-form can be used to write compressed versions. For example, plate_0[3:5]_[a,b,e,f][1:2:11] refers to rows a, b, e, f; odd columns (note the step of 2), in plates 3, 4, and 5." sqref="B2:B1048576" xr:uid="{C31537EB-99C0-F745-8936-5F243E0408C9}"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -553,6 +570,10 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Transformations::Name" prompt="The name of the transformation. It should only contain alphanumeric characters and underscores, starting with a letter." sqref="A2:A1048576" xr:uid="{C8B21174-460F-1742-832C-0CDC18FAE5FE}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Transformations::Equation" prompt="The value of the variable stored in Transformations::Name. Only evaluated when neccessary (when esm views is called and the value of this transformation is required)." sqref="B2:B1048576" xr:uid="{507F27F2-484C-354D-8FC6-607C50B09EEB}"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -571,6 +592,10 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Views::Name" prompt="The name of the view. It should only contain alphanumeric characters and underscores, starting with a letter. This is the name to access the view from esm views." sqref="A2:A1048576" xr:uid="{59485B76-095E-0841-AB11-CD1D36B42731}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Views::View" prompt="What data should be used in the view. Should be a value in one of Transformations::Name, Groups::Name, or a name of a sample (e.g. plate_01_a1)." sqref="B2:B1048576" xr:uid="{56E5700B-8093-2E49-9A2C-34EE722C1011}"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add Samples::Type drop down to template
</commit_message>
<xml_diff>
--- a/src/ESM.xlsx
+++ b/src/ESM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C73AF8C-C2F1-E44B-81B1-8BEB85550543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6338912B-2C87-0742-9042-B8812BF8AAC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
@@ -489,7 +489,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Plate brand" prompt="The brand of plate reader used for the data. If Samples::Type is not plate reader, this can be left blank." sqref="D2:D1048576" xr:uid="{F795587E-0606-8D47-AA35-A77937E6BFD0}">
       <formula1>"BioTek, Tecan, BMG, SpectraMax, Generic"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Type" prompt="The type of experimental data. Either &quot;plate reader&quot; for any plate reader file, or &quot;flow&quot; for flow cytometry fcs files." sqref="A2:A1048576" xr:uid="{CF35B5DA-5768-0E4F-878A-C64AE48DF9B0}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Type" prompt="The type of experimental data. Either &quot;plate reader&quot; for any plate reader file, or &quot;flow&quot; for flow cytometry fcs files." sqref="A2:A1048576" xr:uid="{CF35B5DA-5768-0E4F-878A-C64AE48DF9B0}">
+      <formula1>"plate reader, flow"</formula1>
+    </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Data Location" prompt="The file location of the experimental data. It should either be an absolute file path, or relative to the directory from which esm translate is called. If Samples::Type=&quot;flow&quot;, this can be a directory of fcs files." sqref="B2:B1048576" xr:uid="{C349ED61-BB07-3C40-8A36-DD5340FD2263}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Channels" prompt="The channels to translate into the esm file. Any channels not specified will not be included. If blank, all channels will be included. Available channels can be found with esm summarise. Multiple channels can be provided as a comma-separated list." sqref="C2:C1048576" xr:uid="{551D77D5-3392-5345-AFA9-BEC77E06FD7B}"/>
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Samples::Plate" prompt="The plate number used in ESM to refer to this data. Must be a positive whole number. For example, if Samples::Plate=5, this data can be referred to as the wells of plate_05 in ESM." sqref="E2:E1048576" xr:uid="{107CB822-50EF-4C42-B564-6339739ADB7F}">

</xml_diff>